<commit_message>
feat: migrate hydraulics correlation and batch execution
</commit_message>
<xml_diff>
--- a/workbooks/source/Steady_State_Hydraulics_and_Nozzle_Optimization_SI.xlsx
+++ b/workbooks/source/Steady_State_Hydraulics_and_Nozzle_Optimization_SI.xlsx
@@ -9529,7 +9529,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="41" t="str">
-        <x:v>/analyses/hydraulics/flowPath/*/name</x:v>
+        <x:v>/analyses/hydraulics/minimumAnnularVelocity</x:v>
       </x:c>
       <x:c r="B16" s="41" t="str">
         <x:v>Input</x:v>
@@ -9538,31 +9538,25 @@
         <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D16" s="41" t="str">
-        <x:v>D6:D13</x:v>
+        <x:v>B15</x:v>
       </x:c>
       <x:c r="E16" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F16" s="41" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G16" s="41" t="str">
-        <x:v>I</x:v>
-      </x:c>
-      <x:c r="H16" s="41" t="n">
-        <x:v>8</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F16" s="41" t="str"/>
+      <x:c r="G16" s="41" t="str"/>
+      <x:c r="H16" s="41" t="str"/>
       <x:c r="I16" s="41" t="str">
-        <x:v>text</x:v>
+        <x:v>m/s</x:v>
       </x:c>
       <x:c r="J16" s="41" t="str">
-        <x:v>text</x:v>
+        <x:v>speed</x:v>
       </x:c>
       <x:c r="K16" s="41" t="str">
-        <x:v>string</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="L16" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="44" t="b">
         <x:v>1</x:v>
@@ -9571,7 +9565,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="41" t="str">
-        <x:v>/analyses/hydraulics/flowPath/*/length</x:v>
+        <x:v>/analyses/hydraulics/ecdReferenceTvd</x:v>
       </x:c>
       <x:c r="B17" s="41" t="str">
         <x:v>Input</x:v>
@@ -9580,20 +9574,14 @@
         <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D17" s="41" t="str">
-        <x:v>E6:E13</x:v>
+        <x:v>B16</x:v>
       </x:c>
       <x:c r="E17" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F17" s="41" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G17" s="41" t="str">
-        <x:v>I</x:v>
-      </x:c>
-      <x:c r="H17" s="41" t="n">
-        <x:v>8</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F17" s="41" t="str"/>
+      <x:c r="G17" s="41" t="str"/>
+      <x:c r="H17" s="41" t="str"/>
       <x:c r="I17" s="41" t="str">
         <x:v>m</x:v>
       </x:c>
@@ -9604,7 +9592,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="L17" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M17" s="44" t="b">
         <x:v>1</x:v>
@@ -9613,7 +9601,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="41" t="str">
-        <x:v>/analyses/hydraulics/flowPath/*/flowId</x:v>
+        <x:v>/analyses/hydraulics/surfaceBackpressure</x:v>
       </x:c>
       <x:c r="B18" s="41" t="str">
         <x:v>Input</x:v>
@@ -9622,31 +9610,25 @@
         <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D18" s="41" t="str">
-        <x:v>F6:F13</x:v>
+        <x:v>B17</x:v>
       </x:c>
       <x:c r="E18" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F18" s="41" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G18" s="41" t="str">
-        <x:v>I</x:v>
-      </x:c>
-      <x:c r="H18" s="41" t="n">
-        <x:v>8</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F18" s="41" t="str"/>
+      <x:c r="G18" s="41" t="str"/>
+      <x:c r="H18" s="41" t="str"/>
       <x:c r="I18" s="41" t="str">
-        <x:v>m</x:v>
+        <x:v>Pa</x:v>
       </x:c>
       <x:c r="J18" s="41" t="str">
-        <x:v>length</x:v>
+        <x:v>pressure</x:v>
       </x:c>
       <x:c r="K18" s="41" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="L18" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M18" s="44" t="b">
         <x:v>1</x:v>
@@ -9655,7 +9637,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>/analyses/hydraulics/flowPath/*/flowType</x:v>
+        <x:v>/analyses/hydraulics/pressureCorrelation</x:v>
       </x:c>
       <x:c r="B19" s="41" t="str">
         <x:v>Input</x:v>
@@ -9664,20 +9646,14 @@
         <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D19" s="41" t="str">
-        <x:v>G6:G13</x:v>
+        <x:v>B18</x:v>
       </x:c>
       <x:c r="E19" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>G</x:v>
-      </x:c>
-      <x:c r="G19" s="41" t="str">
-        <x:v>I</x:v>
-      </x:c>
-      <x:c r="H19" s="41" t="n">
-        <x:v>8</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F19" s="41" t="str"/>
+      <x:c r="G19" s="41" t="str"/>
+      <x:c r="H19" s="41" t="str"/>
       <x:c r="I19" s="41" t="str">
         <x:v>text</x:v>
       </x:c>
@@ -9688,7 +9664,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="L19" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M19" s="44" t="b">
         <x:v>1</x:v>
@@ -9697,7 +9673,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="41" t="str">
-        <x:v>/analyses/hydraulics/flowPath/*/hydraulicDiameter</x:v>
+        <x:v>/analyses/hydraulics/computeBackend</x:v>
       </x:c>
       <x:c r="B20" s="41" t="str">
         <x:v>Input</x:v>
@@ -9706,31 +9682,25 @@
         <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D20" s="41" t="str">
-        <x:v>H6:H13</x:v>
+        <x:v>B19</x:v>
       </x:c>
       <x:c r="E20" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F20" s="41" t="str">
-        <x:v>H</x:v>
-      </x:c>
-      <x:c r="G20" s="41" t="str">
-        <x:v>I</x:v>
-      </x:c>
-      <x:c r="H20" s="41" t="n">
-        <x:v>8</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F20" s="41" t="str"/>
+      <x:c r="G20" s="41" t="str"/>
+      <x:c r="H20" s="41" t="str"/>
       <x:c r="I20" s="41" t="str">
-        <x:v>m</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="J20" s="41" t="str">
-        <x:v>diameter</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="K20" s="41" t="str">
-        <x:v>number</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="L20" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M20" s="44" t="b">
         <x:v>1</x:v>
@@ -9739,40 +9709,34 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="41" t="str">
-        <x:v>/pumpNozzle/nozzles/*/diameter</x:v>
+        <x:v>/analyses/hydraulics/thermalAssumption</x:v>
       </x:c>
       <x:c r="B21" s="41" t="str">
         <x:v>Input</x:v>
       </x:c>
       <x:c r="C21" s="41" t="str">
-        <x:v>Calc</x:v>
+        <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D21" s="41" t="str">
-        <x:v>L6:L10</x:v>
+        <x:v>B20</x:v>
       </x:c>
       <x:c r="E21" s="41" t="str">
-        <x:v>Table</x:v>
-      </x:c>
-      <x:c r="F21" s="41" t="str">
-        <x:v>L</x:v>
-      </x:c>
-      <x:c r="G21" s="41" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="H21" s="41" t="n">
-        <x:v>5</x:v>
-      </x:c>
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F21" s="41" t="str"/>
+      <x:c r="G21" s="41" t="str"/>
+      <x:c r="H21" s="41" t="str"/>
       <x:c r="I21" s="41" t="str">
-        <x:v>m</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="J21" s="41" t="str">
-        <x:v>diameter</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="K21" s="41" t="str">
-        <x:v>number</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="L21" s="44" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M21" s="44" t="b">
         <x:v>1</x:v>
@@ -9781,16 +9745,16 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/totalFlowPathLoss</x:v>
+        <x:v>/analyses/hydraulics/rheology/model</x:v>
       </x:c>
       <x:c r="B22" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C22" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D22" s="41" t="str">
-        <x:v>B6</x:v>
+        <x:v>G6</x:v>
       </x:c>
       <x:c r="E22" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9799,34 +9763,34 @@
       <x:c r="G22" s="41" t="str"/>
       <x:c r="H22" s="41" t="str"/>
       <x:c r="I22" s="41" t="str">
-        <x:v>Results!C6</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="J22" s="41" t="str">
-        <x:v>pressure</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="K22" s="41" t="str">
-        <x:v>number</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="L22" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M22" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N22" s="35"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
-        <x:v>/analyses/hydraulics/summary/recommendedNozzleDiameter</x:v>
+        <x:v>/analyses/hydraulics/rheology/flowBehaviorIndex</x:v>
       </x:c>
       <x:c r="B23" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D23" s="41" t="str">
-        <x:v>B7</x:v>
+        <x:v>B8</x:v>
       </x:c>
       <x:c r="E23" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9835,10 +9799,10 @@
       <x:c r="G23" s="41" t="str"/>
       <x:c r="H23" s="41" t="str"/>
       <x:c r="I23" s="41" t="str">
-        <x:v>Results!C7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J23" s="41" t="str">
-        <x:v>diameter</x:v>
+        <x:v>unitless</x:v>
       </x:c>
       <x:c r="K23" s="41" t="str">
         <x:v>number</x:v>
@@ -9847,22 +9811,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M23" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N23" s="35"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/recommendedSurfacePressure</x:v>
+        <x:v>/analyses/hydraulics/rheology/consistencyCoefficient</x:v>
       </x:c>
       <x:c r="B24" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C24" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D24" s="41" t="str">
-        <x:v>B8</x:v>
+        <x:v>B9</x:v>
       </x:c>
       <x:c r="E24" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9871,10 +9835,10 @@
       <x:c r="G24" s="41" t="str"/>
       <x:c r="H24" s="41" t="str"/>
       <x:c r="I24" s="41" t="str">
-        <x:v>Results!C8</x:v>
+        <x:v>Pa*s^n</x:v>
       </x:c>
       <x:c r="J24" s="41" t="str">
-        <x:v>pressure</x:v>
+        <x:v>rheologyConsistency</x:v>
       </x:c>
       <x:c r="K24" s="41" t="str">
         <x:v>number</x:v>
@@ -9883,22 +9847,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N24" s="35"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/nozzleVelocity</x:v>
+        <x:v>/analyses/hydraulics/rheology/yieldStress</x:v>
       </x:c>
       <x:c r="B25" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C25" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D25" s="41" t="str">
-        <x:v>B9</x:v>
+        <x:v>B10</x:v>
       </x:c>
       <x:c r="E25" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9907,10 +9871,10 @@
       <x:c r="G25" s="41" t="str"/>
       <x:c r="H25" s="41" t="str"/>
       <x:c r="I25" s="41" t="str">
-        <x:v>Results!C9</x:v>
+        <x:v>Pa</x:v>
       </x:c>
       <x:c r="J25" s="41" t="str">
-        <x:v>speed</x:v>
+        <x:v>stress</x:v>
       </x:c>
       <x:c r="K25" s="41" t="str">
         <x:v>number</x:v>
@@ -9919,22 +9883,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M25" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N25" s="35"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/ecdScreeningInput</x:v>
+        <x:v>/analyses/hydraulics/rheology/plasticViscosity</x:v>
       </x:c>
       <x:c r="B26" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C26" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D26" s="41" t="str">
-        <x:v>B10</x:v>
+        <x:v>B11</x:v>
       </x:c>
       <x:c r="E26" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9943,10 +9907,10 @@
       <x:c r="G26" s="41" t="str"/>
       <x:c r="H26" s="41" t="str"/>
       <x:c r="I26" s="41" t="str">
-        <x:v>Results!C10</x:v>
+        <x:v>Pa*s</x:v>
       </x:c>
       <x:c r="J26" s="41" t="str">
-        <x:v>density</x:v>
+        <x:v>viscosity</x:v>
       </x:c>
       <x:c r="K26" s="41" t="str">
         <x:v>number</x:v>
@@ -9955,22 +9919,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M26" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N26" s="35"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/flowPathStatus</x:v>
+        <x:v>/analyses/hydraulics/rheology/surfaceTemperature</x:v>
       </x:c>
       <x:c r="B27" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D27" s="41" t="str">
-        <x:v>E6</x:v>
+        <x:v>B12</x:v>
       </x:c>
       <x:c r="E27" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -9979,34 +9943,34 @@
       <x:c r="G27" s="41" t="str"/>
       <x:c r="H27" s="41" t="str"/>
       <x:c r="I27" s="41" t="str">
-        <x:v>text</x:v>
+        <x:v>K</x:v>
       </x:c>
       <x:c r="J27" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>temperature</x:v>
       </x:c>
       <x:c r="K27" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="L27" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M27" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N27" s="35"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/nozzleStatus</x:v>
+        <x:v>/analyses/hydraulics/rheology/compressibility</x:v>
       </x:c>
       <x:c r="B28" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C28" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D28" s="41" t="str">
-        <x:v>E7</x:v>
+        <x:v>B13</x:v>
       </x:c>
       <x:c r="E28" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -10015,34 +9979,34 @@
       <x:c r="G28" s="41" t="str"/>
       <x:c r="H28" s="41" t="str"/>
       <x:c r="I28" s="41" t="str">
-        <x:v>text</x:v>
+        <x:v>1/Pa</x:v>
       </x:c>
       <x:c r="J28" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>compressibility</x:v>
       </x:c>
       <x:c r="K28" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="L28" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M28" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N28" s="35"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="41" t="str">
-        <x:v>/analyses/hydraulics/summary/surfacePressureStatus</x:v>
+        <x:v>/analyses/hydraulics/rheology/highShearFlowIndex</x:v>
       </x:c>
       <x:c r="B29" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C29" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Fluid Model</x:v>
       </x:c>
       <x:c r="D29" s="41" t="str">
-        <x:v>E8</x:v>
+        <x:v>B14</x:v>
       </x:c>
       <x:c r="E29" s="41" t="str">
         <x:v>Scalar</x:v>
@@ -10051,93 +10015,633 @@
       <x:c r="G29" s="41" t="str"/>
       <x:c r="H29" s="41" t="str"/>
       <x:c r="I29" s="41" t="str">
-        <x:v>text</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J29" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>unitless</x:v>
       </x:c>
       <x:c r="K29" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="L29" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M29" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N29" s="35"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="41" t="str">
-        <x:v>/analyses/hydraulics/results/nozzleVelocityStatus</x:v>
+        <x:v>/analyses/hydraulics/flowPath/*/name</x:v>
       </x:c>
       <x:c r="B30" s="41" t="str">
-        <x:v>Output</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="C30" s="41" t="str">
-        <x:v>Results</x:v>
+        <x:v>Inputs</x:v>
       </x:c>
       <x:c r="D30" s="41" t="str">
-        <x:v>E9</x:v>
+        <x:v>D6:D13</x:v>
       </x:c>
       <x:c r="E30" s="41" t="str">
-        <x:v>Scalar</x:v>
-      </x:c>
-      <x:c r="F30" s="41" t="str"/>
-      <x:c r="G30" s="41" t="str"/>
-      <x:c r="H30" s="41" t="str"/>
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F30" s="41" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G30" s="41" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="H30" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="I30" s="41" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="J30" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="K30" s="41" t="str">
-        <x:v>status</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="L30" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M30" s="44" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N30" s="35"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="41" t="str">
+        <x:v>/analyses/hydraulics/flowPath/*/length</x:v>
+      </x:c>
+      <x:c r="B31" s="41" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="C31" s="41" t="str">
+        <x:v>Inputs</x:v>
+      </x:c>
+      <x:c r="D31" s="41" t="str">
+        <x:v>E6:E13</x:v>
+      </x:c>
+      <x:c r="E31" s="41" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F31" s="41" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G31" s="41" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="H31" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I31" s="41" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="J31" s="41" t="str">
+        <x:v>length</x:v>
+      </x:c>
+      <x:c r="K31" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L31" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M31" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N31" s="35"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="41" t="str">
+        <x:v>/analyses/hydraulics/flowPath/*/flowId</x:v>
+      </x:c>
+      <x:c r="B32" s="41" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="C32" s="41" t="str">
+        <x:v>Inputs</x:v>
+      </x:c>
+      <x:c r="D32" s="41" t="str">
+        <x:v>F6:F13</x:v>
+      </x:c>
+      <x:c r="E32" s="41" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F32" s="41" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G32" s="41" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="H32" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I32" s="41" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="J32" s="41" t="str">
+        <x:v>length</x:v>
+      </x:c>
+      <x:c r="K32" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L32" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M32" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N32" s="35"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="41" t="str">
+        <x:v>/analyses/hydraulics/flowPath/*/flowType</x:v>
+      </x:c>
+      <x:c r="B33" s="41" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="C33" s="41" t="str">
+        <x:v>Inputs</x:v>
+      </x:c>
+      <x:c r="D33" s="41" t="str">
+        <x:v>G6:G13</x:v>
+      </x:c>
+      <x:c r="E33" s="41" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F33" s="41" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="G33" s="41" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="H33" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I33" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="J33" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="K33" s="41" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="L33" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M33" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N33" s="35"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="41" t="str">
+        <x:v>/analyses/hydraulics/flowPath/*/hydraulicDiameter</x:v>
+      </x:c>
+      <x:c r="B34" s="41" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="C34" s="41" t="str">
+        <x:v>Inputs</x:v>
+      </x:c>
+      <x:c r="D34" s="41" t="str">
+        <x:v>H6:H13</x:v>
+      </x:c>
+      <x:c r="E34" s="41" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F34" s="41" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="G34" s="41" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="H34" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I34" s="41" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="J34" s="41" t="str">
+        <x:v>diameter</x:v>
+      </x:c>
+      <x:c r="K34" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L34" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M34" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N34" s="35"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="41" t="str">
+        <x:v>/pumpNozzle/nozzles/*/diameter</x:v>
+      </x:c>
+      <x:c r="B35" s="41" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="C35" s="41" t="str">
+        <x:v>Calc</x:v>
+      </x:c>
+      <x:c r="D35" s="41" t="str">
+        <x:v>L6:L10</x:v>
+      </x:c>
+      <x:c r="E35" s="41" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="F35" s="41" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="G35" s="41" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="H35" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I35" s="41" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="J35" s="41" t="str">
+        <x:v>diameter</x:v>
+      </x:c>
+      <x:c r="K35" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L35" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M35" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N35" s="35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/totalFlowPathLoss</x:v>
+      </x:c>
+      <x:c r="B36" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C36" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D36" s="41" t="str">
+        <x:v>B6</x:v>
+      </x:c>
+      <x:c r="E36" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F36" s="41" t="str"/>
+      <x:c r="G36" s="41" t="str"/>
+      <x:c r="H36" s="41" t="str"/>
+      <x:c r="I36" s="41" t="str">
+        <x:v>Results!C6</x:v>
+      </x:c>
+      <x:c r="J36" s="41" t="str">
+        <x:v>pressure</x:v>
+      </x:c>
+      <x:c r="K36" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L36" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="35"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="41" t="str">
+        <x:v>/analyses/hydraulics/summary/recommendedNozzleDiameter</x:v>
+      </x:c>
+      <x:c r="B37" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C37" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D37" s="41" t="str">
+        <x:v>B7</x:v>
+      </x:c>
+      <x:c r="E37" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F37" s="41" t="str"/>
+      <x:c r="G37" s="41" t="str"/>
+      <x:c r="H37" s="41" t="str"/>
+      <x:c r="I37" s="41" t="str">
+        <x:v>Results!C7</x:v>
+      </x:c>
+      <x:c r="J37" s="41" t="str">
+        <x:v>diameter</x:v>
+      </x:c>
+      <x:c r="K37" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L37" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="35"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/recommendedSurfacePressure</x:v>
+      </x:c>
+      <x:c r="B38" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C38" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D38" s="41" t="str">
+        <x:v>B8</x:v>
+      </x:c>
+      <x:c r="E38" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F38" s="41" t="str"/>
+      <x:c r="G38" s="41" t="str"/>
+      <x:c r="H38" s="41" t="str"/>
+      <x:c r="I38" s="41" t="str">
+        <x:v>Results!C8</x:v>
+      </x:c>
+      <x:c r="J38" s="41" t="str">
+        <x:v>pressure</x:v>
+      </x:c>
+      <x:c r="K38" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L38" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="35"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/nozzleVelocity</x:v>
+      </x:c>
+      <x:c r="B39" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C39" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D39" s="41" t="str">
+        <x:v>B9</x:v>
+      </x:c>
+      <x:c r="E39" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F39" s="41" t="str"/>
+      <x:c r="G39" s="41" t="str"/>
+      <x:c r="H39" s="41" t="str"/>
+      <x:c r="I39" s="41" t="str">
+        <x:v>Results!C9</x:v>
+      </x:c>
+      <x:c r="J39" s="41" t="str">
+        <x:v>speed</x:v>
+      </x:c>
+      <x:c r="K39" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L39" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="35"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/ecdScreeningInput</x:v>
+      </x:c>
+      <x:c r="B40" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C40" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D40" s="41" t="str">
+        <x:v>B10</x:v>
+      </x:c>
+      <x:c r="E40" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F40" s="41" t="str"/>
+      <x:c r="G40" s="41" t="str"/>
+      <x:c r="H40" s="41" t="str"/>
+      <x:c r="I40" s="41" t="str">
+        <x:v>Results!C10</x:v>
+      </x:c>
+      <x:c r="J40" s="41" t="str">
+        <x:v>density</x:v>
+      </x:c>
+      <x:c r="K40" s="41" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="L40" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M40" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="35"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/flowPathStatus</x:v>
+      </x:c>
+      <x:c r="B41" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C41" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D41" s="41" t="str">
+        <x:v>E6</x:v>
+      </x:c>
+      <x:c r="E41" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F41" s="41" t="str"/>
+      <x:c r="G41" s="41" t="str"/>
+      <x:c r="H41" s="41" t="str"/>
+      <x:c r="I41" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="J41" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="K41" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="L41" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M41" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="35"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/nozzleStatus</x:v>
+      </x:c>
+      <x:c r="B42" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C42" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D42" s="41" t="str">
+        <x:v>E7</x:v>
+      </x:c>
+      <x:c r="E42" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F42" s="41" t="str"/>
+      <x:c r="G42" s="41" t="str"/>
+      <x:c r="H42" s="41" t="str"/>
+      <x:c r="I42" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="J42" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="K42" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="L42" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M42" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="35"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="41" t="str">
+        <x:v>/analyses/hydraulics/summary/surfacePressureStatus</x:v>
+      </x:c>
+      <x:c r="B43" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C43" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D43" s="41" t="str">
+        <x:v>E8</x:v>
+      </x:c>
+      <x:c r="E43" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F43" s="41" t="str"/>
+      <x:c r="G43" s="41" t="str"/>
+      <x:c r="H43" s="41" t="str"/>
+      <x:c r="I43" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="J43" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="K43" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="L43" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M43" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="35"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="41" t="str">
+        <x:v>/analyses/hydraulics/results/nozzleVelocityStatus</x:v>
+      </x:c>
+      <x:c r="B44" s="41" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="C44" s="41" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="D44" s="41" t="str">
+        <x:v>E9</x:v>
+      </x:c>
+      <x:c r="E44" s="41" t="str">
+        <x:v>Scalar</x:v>
+      </x:c>
+      <x:c r="F44" s="41" t="str"/>
+      <x:c r="G44" s="41" t="str"/>
+      <x:c r="H44" s="41" t="str"/>
+      <x:c r="I44" s="41" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="J44" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="K44" s="41" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="L44" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M44" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="35"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="41" t="str">
         <x:v>/analyses/hydraulics/results/ecdStatus</x:v>
       </x:c>
-      <x:c r="B31" s="41" t="str">
+      <x:c r="B45" s="41" t="str">
         <x:v>Output</x:v>
       </x:c>
-      <x:c r="C31" s="41" t="str">
+      <x:c r="C45" s="41" t="str">
         <x:v>Results</x:v>
       </x:c>
-      <x:c r="D31" s="41" t="str">
+      <x:c r="D45" s="41" t="str">
         <x:v>E10</x:v>
       </x:c>
-      <x:c r="E31" s="41" t="str">
+      <x:c r="E45" s="41" t="str">
         <x:v>Scalar</x:v>
       </x:c>
-      <x:c r="F31" s="41" t="str"/>
-      <x:c r="G31" s="41" t="str"/>
-      <x:c r="H31" s="41" t="str"/>
-      <x:c r="I31" s="41" t="str">
+      <x:c r="F45" s="41" t="str"/>
+      <x:c r="G45" s="41" t="str"/>
+      <x:c r="H45" s="41" t="str"/>
+      <x:c r="I45" s="41" t="str">
         <x:v>text</x:v>
       </x:c>
-      <x:c r="J31" s="41" t="str">
+      <x:c r="J45" s="41" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="K31" s="41" t="str">
+      <x:c r="K45" s="41" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="L31" s="44" t="b">
+      <x:c r="L45" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M31" s="44" t="b">
+      <x:c r="M45" s="44" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N31" s="35"/>
+      <x:c r="N45" s="35"/>
     </x:row>
   </x:sheetData>
   <x:sheetProtection sheet="1" objects="1" scenarios="1"/>
@@ -10891,11 +11395,122 @@
       <x:c r="M15" s="35"/>
       <x:c r="N15" s="35"/>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="35" t="str">
+        <x:v>ECD reference TVD m</x:v>
+      </x:c>
+      <x:c r="B16" s="39" t="n">
+        <x:v>2660</x:v>
+      </x:c>
+      <x:c r="C16" s="35"/>
+      <x:c r="D16" s="35"/>
+      <x:c r="E16" s="35"/>
+      <x:c r="F16" s="35"/>
+      <x:c r="G16" s="35"/>
+      <x:c r="H16" s="35"/>
+      <x:c r="I16" s="35"/>
+      <x:c r="J16" s="35"/>
+      <x:c r="K16" s="35"/>
+      <x:c r="L16" s="35"/>
+      <x:c r="M16" s="35"/>
+      <x:c r="N16" s="35"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="35" t="str">
+        <x:v>Surface backpressure Pa</x:v>
+      </x:c>
+      <x:c r="B17" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="35"/>
+      <x:c r="D17" s="35"/>
+      <x:c r="E17" s="35"/>
+      <x:c r="F17" s="35"/>
+      <x:c r="G17" s="35"/>
+      <x:c r="H17" s="35"/>
+      <x:c r="I17" s="35"/>
+      <x:c r="J17" s="35"/>
+      <x:c r="K17" s="35"/>
+      <x:c r="L17" s="35"/>
+      <x:c r="M17" s="35"/>
+      <x:c r="N17" s="35"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="35" t="str">
+        <x:v>Pressure correlation</x:v>
+      </x:c>
+      <x:c r="B18" s="39" t="str">
+        <x:v>darcy_weisbach_screening</x:v>
+      </x:c>
+      <x:c r="C18" s="35"/>
+      <x:c r="D18" s="35"/>
+      <x:c r="E18" s="35"/>
+      <x:c r="F18" s="35"/>
+      <x:c r="G18" s="35"/>
+      <x:c r="H18" s="35"/>
+      <x:c r="I18" s="35"/>
+      <x:c r="J18" s="35"/>
+      <x:c r="K18" s="35"/>
+      <x:c r="L18" s="35"/>
+      <x:c r="M18" s="35"/>
+      <x:c r="N18" s="35"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="35" t="str">
+        <x:v>Compute backend</x:v>
+      </x:c>
+      <x:c r="B19" s="39" t="str">
+        <x:v>serial_cpu</x:v>
+      </x:c>
+      <x:c r="C19" s="35"/>
+      <x:c r="D19" s="35"/>
+      <x:c r="E19" s="35"/>
+      <x:c r="F19" s="35"/>
+      <x:c r="G19" s="35"/>
+      <x:c r="H19" s="35"/>
+      <x:c r="I19" s="35"/>
+      <x:c r="J19" s="35"/>
+      <x:c r="K19" s="35"/>
+      <x:c r="L19" s="35"/>
+      <x:c r="M19" s="35"/>
+      <x:c r="N19" s="35"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="35" t="str">
+        <x:v>Thermal assumption</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="str">
+        <x:v>constant_properties</x:v>
+      </x:c>
+      <x:c r="C20" s="35"/>
+      <x:c r="D20" s="35"/>
+      <x:c r="E20" s="35"/>
+      <x:c r="F20" s="35"/>
+      <x:c r="G20" s="35"/>
+      <x:c r="H20" s="35"/>
+      <x:c r="I20" s="35"/>
+      <x:c r="J20" s="35"/>
+      <x:c r="K20" s="35"/>
+      <x:c r="L20" s="35"/>
+      <x:c r="M20" s="35"/>
+      <x:c r="N20" s="35"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="B18">
+      <x:formula1>"generalized_yield_power_law,darcy_weisbach_screening"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B19">
+      <x:formula1>"parallel_cpu,serial_cpu"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B20">
+      <x:formula1>"constant_properties"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -12327,13 +12942,13 @@
       </x:c>
       <x:c r="E5" s="35"/>
       <x:c r="F5" s="36" t="str">
-        <x:v>Model</x:v>
+        <x:v>Control</x:v>
       </x:c>
       <x:c r="G5" s="36" t="str">
-        <x:v>Selected</x:v>
+        <x:v>Value</x:v>
       </x:c>
       <x:c r="H5" s="36" t="str">
-        <x:v>Applicability</x:v>
+        <x:v>Purpose</x:v>
       </x:c>
       <x:c r="I5" s="35"/>
       <x:c r="J5" s="35"/>
@@ -12347,6 +12962,7 @@
         <x:v>Mud density</x:v>
       </x:c>
       <x:c r="B6" s="39" t="n">
+        <x:f>Inputs!B9</x:f>
         <x:v>1200</x:v>
       </x:c>
       <x:c r="C6" s="35" t="str">
@@ -12357,13 +12973,13 @@
       </x:c>
       <x:c r="E6" s="35"/>
       <x:c r="F6" s="35" t="str">
-        <x:v>Newtonian</x:v>
+        <x:v>Constitutive model</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
-        <x:v>No</x:v>
+        <x:v>power_law</x:v>
       </x:c>
       <x:c r="H6" s="35" t="str">
-        <x:v>Initial screening</x:v>
+        <x:v>Rust contract enum</x:v>
       </x:c>
       <x:c r="I6" s="35"/>
       <x:c r="J6" s="35"/>
@@ -12374,27 +12990,22 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="35" t="str">
-        <x:v>Apparent viscosity</x:v>
+        <x:v>Dynamic viscosity</x:v>
       </x:c>
       <x:c r="B7" s="39" t="n">
+        <x:f>Inputs!B10</x:f>
         <x:v>0.035</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
-        <x:v>Pa-s</x:v>
+        <x:v>Pa*s</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
-        <x:v>Newtonian screen</x:v>
+        <x:v>Newtonian model</x:v>
       </x:c>
       <x:c r="E7" s="35"/>
-      <x:c r="F7" s="35" t="str">
-        <x:v>Power law</x:v>
-      </x:c>
-      <x:c r="G7" s="39" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H7" s="35" t="str">
-        <x:v>Section pressure loss</x:v>
-      </x:c>
+      <x:c r="F7" s="35"/>
+      <x:c r="G7" s="35"/>
+      <x:c r="H7" s="35"/>
       <x:c r="I7" s="35"/>
       <x:c r="J7" s="35"/>
       <x:c r="K7" s="35"/>
@@ -12410,20 +13021,20 @@
         <x:v>0.72</x:v>
       </x:c>
       <x:c r="C8" s="35" t="str">
-        <x:v>fraction</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
-        <x:v>Power-law exponent</x:v>
+        <x:v>Yield-power-law exponent</x:v>
       </x:c>
       <x:c r="E8" s="35"/>
-      <x:c r="F8" s="35" t="str">
-        <x:v>Bingham plastic</x:v>
-      </x:c>
-      <x:c r="G8" s="39" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="H8" s="35" t="str">
-        <x:v>Cross-check</x:v>
+      <x:c r="F8" s="36" t="str">
+        <x:v>Model</x:v>
+      </x:c>
+      <x:c r="G8" s="36" t="str">
+        <x:v>Required SI parameters</x:v>
+      </x:c>
+      <x:c r="H8" s="36" t="str">
+        <x:v>Use</x:v>
       </x:c>
       <x:c r="I8" s="35"/>
       <x:c r="J8" s="35"/>
@@ -12434,21 +13045,27 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
-        <x:v>Consistency index</x:v>
+        <x:v>Consistency coefficient</x:v>
       </x:c>
       <x:c r="B9" s="39" t="n">
         <x:v>0.32</x:v>
       </x:c>
       <x:c r="C9" s="35" t="str">
-        <x:v>Pa-s^n</x:v>
+        <x:v>Pa*s^n</x:v>
       </x:c>
       <x:c r="D9" s="35" t="str">
-        <x:v>Power-law consistency</x:v>
+        <x:v>Yield-power-law consistency</x:v>
       </x:c>
       <x:c r="E9" s="35"/>
-      <x:c r="F9" s="35"/>
-      <x:c r="G9" s="35"/>
-      <x:c r="H9" s="35"/>
+      <x:c r="F9" s="35" t="str">
+        <x:v>newtonian</x:v>
+      </x:c>
+      <x:c r="G9" s="35" t="str">
+        <x:v>dynamic viscosity</x:v>
+      </x:c>
+      <x:c r="H9" s="35" t="str">
+        <x:v>Linear viscous fluid</x:v>
+      </x:c>
       <x:c r="I9" s="35"/>
       <x:c r="J9" s="35"/>
       <x:c r="K9" s="35"/>
@@ -12458,7 +13075,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
-        <x:v>Yield point</x:v>
+        <x:v>Yield stress</x:v>
       </x:c>
       <x:c r="B10" s="39" t="n">
         <x:v>8.5</x:v>
@@ -12467,12 +13084,18 @@
         <x:v>Pa</x:v>
       </x:c>
       <x:c r="D10" s="35" t="str">
-        <x:v>Herschel-Bulkley screen</x:v>
+        <x:v>Bingham and Herschel-Bulkley</x:v>
       </x:c>
       <x:c r="E10" s="35"/>
-      <x:c r="F10" s="35"/>
-      <x:c r="G10" s="35"/>
-      <x:c r="H10" s="35"/>
+      <x:c r="F10" s="35" t="str">
+        <x:v>power_law</x:v>
+      </x:c>
+      <x:c r="G10" s="35" t="str">
+        <x:v>consistency, flow index, high-shear index</x:v>
+      </x:c>
+      <x:c r="H10" s="35" t="str">
+        <x:v>Shear-dependent fluid</x:v>
+      </x:c>
       <x:c r="I10" s="35"/>
       <x:c r="J10" s="35"/>
       <x:c r="K10" s="35"/>
@@ -12488,15 +13111,21 @@
         <x:v>0.024</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>Pa-s</x:v>
+        <x:v>Pa*s</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>Bingham screen</x:v>
+        <x:v>Bingham model</x:v>
       </x:c>
       <x:c r="E11" s="35"/>
-      <x:c r="F11" s="35"/>
-      <x:c r="G11" s="35"/>
-      <x:c r="H11" s="35"/>
+      <x:c r="F11" s="35" t="str">
+        <x:v>bingham</x:v>
+      </x:c>
+      <x:c r="G11" s="35" t="str">
+        <x:v>yield stress, plastic viscosity</x:v>
+      </x:c>
+      <x:c r="H11" s="35" t="str">
+        <x:v>Linear post-yield fluid</x:v>
+      </x:c>
       <x:c r="I11" s="35"/>
       <x:c r="J11" s="35"/>
       <x:c r="K11" s="35"/>
@@ -12506,7 +13135,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="35" t="str">
-        <x:v>Temperature</x:v>
+        <x:v>Surface temperature</x:v>
       </x:c>
       <x:c r="B12" s="39" t="n">
         <x:v>333.15</x:v>
@@ -12515,12 +13144,18 @@
         <x:v>K</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>Reference condition</x:v>
+        <x:v>Hydraulics reference condition</x:v>
       </x:c>
       <x:c r="E12" s="35"/>
-      <x:c r="F12" s="35"/>
-      <x:c r="G12" s="35"/>
-      <x:c r="H12" s="35"/>
+      <x:c r="F12" s="35" t="str">
+        <x:v>herschel_bulkley</x:v>
+      </x:c>
+      <x:c r="G12" s="35" t="str">
+        <x:v>yield stress, consistency, flow index, high-shear index</x:v>
+      </x:c>
+      <x:c r="H12" s="35" t="str">
+        <x:v>General yield-power-law fluid</x:v>
+      </x:c>
       <x:c r="I12" s="35"/>
       <x:c r="J12" s="35"/>
       <x:c r="K12" s="35"/>
@@ -12539,7 +13174,7 @@
         <x:v>1/Pa</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
-        <x:v>Screening input</x:v>
+        <x:v>Reserved thermal coupling input</x:v>
       </x:c>
       <x:c r="E13" s="35"/>
       <x:c r="F13" s="35"/>
@@ -12552,11 +13187,40 @@
       <x:c r="M13" s="35"/>
       <x:c r="N13" s="35"/>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="35" t="str">
+        <x:v>High-shear flow index</x:v>
+      </x:c>
+      <x:c r="B14" s="39" t="n">
+        <x:v>0.72</x:v>
+      </x:c>
+      <x:c r="C14" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="str">
+        <x:v>Independent turbulent fit</x:v>
+      </x:c>
+      <x:c r="E14" s="35"/>
+      <x:c r="F14" s="35"/>
+      <x:c r="G14" s="35"/>
+      <x:c r="H14" s="35"/>
+      <x:c r="I14" s="35"/>
+      <x:c r="J14" s="35"/>
+      <x:c r="K14" s="35"/>
+      <x:c r="L14" s="35"/>
+      <x:c r="M14" s="35"/>
+      <x:c r="N14" s="35"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G6">
+      <x:formula1>"newtonian,power_law,bingham,herschel_bulkley"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>